<commit_message>
improve template help wording
</commit_message>
<xml_diff>
--- a/vocexcel/templates/VocExcel-template-100-GA.xlsx
+++ b/vocexcel/templates/VocExcel-template-100-GA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/work/kurrawong/VocExcel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/work/kurrawong/VocExcel/vocexcel/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3723E494-BB75-CA4A-B0E6-312951AC5E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B37474-07B2-8745-AFFF-E13D4AB5D990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44840" yWindow="1000" windowWidth="53660" windowHeight="27680" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1789,11 +1789,6 @@
     <t>Broader Concept IRI</t>
   </si>
   <si>
-    <t xml:space="preserve">Select the IRI of a concept that is the broader (parent) concept of this one.
-Concepts that have no broader concept indicated are assumed to be top concepts of the vocabulary.
-If you want multiple parents for a Concept, </t>
-  </si>
-  <si>
     <t>Additional Broader Concept IRI</t>
   </si>
   <si>
@@ -1817,6 +1812,11 @@
   </si>
   <si>
     <t>https://pid.geoscience.gov.au/dataset/ga/</t>
+  </si>
+  <si>
+    <t>Select the IRI of a concept that is the broader (parent) concept of this one.
+Concepts that have no broader concept indicated are assumed to be top concepts of the vocabulary.
+If you want multiple parents for a Concept, add the second and subsequent parents to the Additional Concept Properties sheet</t>
   </si>
 </sst>
 </file>
@@ -2269,6 +2269,9 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2283,9 +2286,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4269,12 +4269,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25" x14ac:dyDescent="0.15">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:4" s="35" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
@@ -4294,8 +4294,8 @@
       <c r="A3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="68" t="s">
-        <v>234</v>
+      <c r="B3" s="63" t="s">
+        <v>233</v>
       </c>
       <c r="C3" s="33" t="s">
         <v>50</v>
@@ -4482,8 +4482,8 @@
       <c r="A18" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="B18" s="68" t="s">
-        <v>235</v>
+      <c r="B18" s="63" t="s">
+        <v>234</v>
       </c>
       <c r="C18" s="33" t="s">
         <v>226</v>
@@ -7500,16 +7500,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.15">
       <c r="A2" s="31" t="s">
@@ -7563,7 +7563,7 @@
         <v>105</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="F3" s="26" t="s">
         <v>130</v>
@@ -10765,16 +10765,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="53" t="s">
@@ -10802,12 +10802,12 @@
         <v>117</v>
       </c>
       <c r="I2" s="54" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:27" s="20" customFormat="1" ht="273" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="26" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>150</v>
@@ -10831,7 +10831,7 @@
         <v>115</v>
       </c>
       <c r="I3" s="45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J3" s="46"/>
       <c r="K3" s="46"/>
@@ -20890,13 +20890,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
     </row>
     <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
@@ -20924,10 +20924,10 @@
         <v>129</v>
       </c>
       <c r="D3" s="50" t="s">
+        <v>231</v>
+      </c>
+      <c r="E3" s="50" t="s">
         <v>232</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="20" customFormat="1" ht="18" x14ac:dyDescent="0.15">
@@ -22275,11 +22275,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
     </row>
     <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="24" t="s">
@@ -22380,11 +22380,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25" x14ac:dyDescent="0.2">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
     </row>
     <row r="2" spans="1:4" ht="21" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
@@ -22631,6 +22631,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006CE8352A0AF1CD4AB9B3521FB05BB06E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ad776eddaa4c2424eb5fa9eef7239753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bcd33c6e-30cb-4633-b8ec-d716de95c77b" xmlns:ns3="cc9fd5b5-cf46-4eda-9201-7118bc1c1603" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c03cb13ad1de5dce1c8a6420670aeaf6" ns2:_="" ns3:_="">
     <xsd:import namespace="bcd33c6e-30cb-4633-b8ec-d716de95c77b"/>
@@ -22867,16 +22876,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41C0741D-72E1-4141-9700-3202E4B56A5A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35C5B03A-DD20-4DDE-9069-342AD74757E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22893,12 +22901,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41C0741D-72E1-4141-9700-3202E4B56A5A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>